<commit_message>
D6 for table 2 created
</commit_message>
<xml_diff>
--- a/i_test/test_D6_Table_S1/g_output/D6_Table_S1_attrition_darolu.xlsx
+++ b/i_test/test_D6_Table_S1/g_output/D6_Table_S1_attrition_darolu.xlsx
@@ -502,7 +502,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>292 (5,8%)</t>
+          <t>292 (34,7%)</t>
         </is>
       </c>
     </row>
@@ -514,7 +514,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>289 (5,8%)</t>
+          <t>289 (34,3%)</t>
         </is>
       </c>
     </row>
@@ -526,7 +526,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>261 (5,2%)</t>
+          <t>261 (31,0%)</t>
         </is>
       </c>
     </row>

</xml_diff>